<commit_message>
Initial draft of everything, file paths rearranged and added main.py.
</commit_message>
<xml_diff>
--- a/output/Tuva_Strategic_Radar_Final.xlsx
+++ b/output/Tuva_Strategic_Radar_Final.xlsx
@@ -16,25 +16,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="152">
   <si>
-    <t>pi_name</t>
-  </si>
-  <si>
-    <t>organization</t>
-  </si>
-  <si>
-    <t>project_title</t>
-  </si>
-  <si>
-    <t>award_amount</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>award_date</t>
-  </si>
-  <si>
-    <t>abstract</t>
+    <t>Pi Name</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>Project Title</t>
+  </si>
+  <si>
+    <t>Award Amount</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>Award Date</t>
+  </si>
+  <si>
+    <t>Abstract</t>
   </si>
   <si>
     <t>ABRAHAMS, VIKKI M</t>
@@ -313,22 +313,22 @@
     <t>Surveillance to track and characterize antimalarial resistance trends in Ugandan Plasmodium falciparum parasites (STARTUP)</t>
   </si>
   <si>
-    <t>2026-02-13T00:00:00</t>
-  </si>
-  <si>
-    <t>2026-02-09T00:00:00</t>
-  </si>
-  <si>
-    <t>2026-02-11T00:00:00</t>
-  </si>
-  <si>
-    <t>2026-02-10T00:00:00</t>
-  </si>
-  <si>
-    <t>2026-02-12T00:00:00</t>
-  </si>
-  <si>
-    <t>2026-02-06T00:00:00</t>
+    <t>2026-02-13</t>
+  </si>
+  <si>
+    <t>2026-02-09</t>
+  </si>
+  <si>
+    <t>2026-02-11</t>
+  </si>
+  <si>
+    <t>2026-02-10</t>
+  </si>
+  <si>
+    <t>2026-02-12</t>
+  </si>
+  <si>
+    <t>2026-02-06</t>
   </si>
   <si>
     <t>Summary/Abstract
@@ -1952,7 +1952,7 @@
     <col min="3" max="3" width="50.7109375" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="5" width="nan" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
     <col min="7" max="7" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>